<commit_message>
Adicionado o arquivo ainda vazio pos_processamento.py
</commit_message>
<xml_diff>
--- a/data/auxiliar_venda.xlsx
+++ b/data/auxiliar_venda.xlsx
@@ -1,31 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\dig_convenios\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6118BFE9-B08A-4B36-B0DC-1C9F8852B918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D6AFA0-5E30-42B9-BBBE-0D05DA25F19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="6">
   <si>
     <t>ACORDO</t>
   </si>
@@ -38,12 +52,21 @@
   <si>
     <t>MES</t>
   </si>
+  <si>
+    <t>CAMPO</t>
+  </si>
+  <si>
+    <t>VALOR</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -53,6 +76,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -75,13 +105,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -95,6 +134,118 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="JANEIRO"/>
+      <sheetName val="FEVEREIRO"/>
+      <sheetName val="MARÇO"/>
+      <sheetName val="ABRIL"/>
+      <sheetName val="MAIO"/>
+      <sheetName val="JUNHO"/>
+      <sheetName val="JULHO"/>
+      <sheetName val="AGOSTO"/>
+      <sheetName val="SETEMBRO"/>
+      <sheetName val="OUTUBRO"/>
+      <sheetName val="NOVEMBRO"/>
+      <sheetName val="DEZEMBRO"/>
+      <sheetName val="TOTAL"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="5">
+          <cell r="C5">
+            <v>72162.5</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1">
+        <row r="5">
+          <cell r="C5">
+            <v>172252.5</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2">
+        <row r="5">
+          <cell r="C5">
+            <v>149190</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="3">
+        <row r="5">
+          <cell r="C5">
+            <v>176858</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="4">
+        <row r="5">
+          <cell r="C5">
+            <v>248230.9</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="5">
+        <row r="5">
+          <cell r="C5">
+            <v>121060.31</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="6">
+        <row r="5">
+          <cell r="C5">
+            <v>250150.25</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="7">
+        <row r="5">
+          <cell r="C5">
+            <v>148438.62</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="8">
+        <row r="5">
+          <cell r="C5">
+            <v>130853.52</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="9">
+        <row r="5">
+          <cell r="C5">
+            <v>141992.93</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="10">
+        <row r="5">
+          <cell r="C5">
+            <v>134999</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="11">
+        <row r="5">
+          <cell r="C5">
+            <v>354411.85</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="12"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -360,155 +511,207 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="13" width="11.7109375" customWidth="1"/>
+    <col min="2" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="12" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>1000</v>
-      </c>
-      <c r="C2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3">
+        <f>[1]JANEIRO!$C$5</f>
+        <v>72162.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3">
-        <v>1001</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3">
+        <f>[1]FEVEREIRO!$C$5</f>
+        <v>172252.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4">
-        <v>1002</v>
-      </c>
-      <c r="C4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3">
+        <f>[1]MARÇO!$C$5</f>
+        <v>149190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5">
-        <v>1003</v>
-      </c>
-      <c r="C5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3">
+        <f>[1]ABRIL!$C$5</f>
+        <v>176858</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
       <c r="B6">
-        <v>1004</v>
-      </c>
-      <c r="C6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="3">
+        <f>[1]MAIO!$C$5</f>
+        <v>248230.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
       <c r="B7">
-        <v>1005</v>
-      </c>
-      <c r="C7">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="3">
+        <f>[1]JUNHO!$C$5</f>
+        <v>121060.31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
       <c r="B8">
-        <v>1006</v>
-      </c>
-      <c r="C8">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="3">
+        <f>[1]JULHO!$C$5</f>
+        <v>250150.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
       <c r="B9">
-        <v>1007</v>
-      </c>
-      <c r="C9">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3">
+        <f>[1]AGOSTO!$C$5</f>
+        <v>148438.62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10">
-        <v>1008</v>
-      </c>
-      <c r="C10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="3">
+        <f>[1]SETEMBRO!$C$5</f>
+        <v>130853.52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
       <c r="B11">
-        <v>1009</v>
-      </c>
-      <c r="C11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3">
+        <f>[1]OUTUBRO!$C$5</f>
+        <v>141992.93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
       <c r="B12">
-        <v>1010</v>
-      </c>
-      <c r="C12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="3">
+        <f>[1]NOVEMBRO!$C$5</f>
+        <v>134999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
       <c r="B13">
-        <v>1011</v>
-      </c>
-      <c r="C13">
         <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3">
+        <f>[1]DEZEMBRO!$C$5</f>
+        <v>354411.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>